<commit_message>
fix: add Release key to STG and UAT sheets in Environment.xlsx
QraceHelper._load_env_excel() calls env_data.get("Release", "") but the
key was missing from both sheets, causing release_name to always be empty
string from default rather than a real lookup. Added Release row with
empty value for QA to fill in the actual build version.

LA_HOSTNAME left as CATHLA01.TH.INTRANE — source artifact
(Qrace Artifacts/Environment Confiig/Enviroment Details.xlsx) has the
same truncated value, so no change was made.
</commit_message>
<xml_diff>
--- a/Config/Environment.xlsx
+++ b/Config/Environment.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -824,6 +824,14 @@
           <t>http://localhost:4444wd/hub</t>
         </is>
       </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -836,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1235,6 +1243,14 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>